<commit_message>
ver 0.4.1.2 minor correction
</commit_message>
<xml_diff>
--- a/data/chapter17_datetime.xlsx
+++ b/data/chapter17_datetime.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kyowapharma-my.sharepoint.com/personal/araya-t_kyowayakuhin_co_jp/Documents/R_scripts/R入門/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\R入門\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="13_ncr:1_{3918B8F2-0D17-40F5-A765-D4D59FEFB31A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37ABDDC4-FC37-4A56-8C6C-80B38C115A7D}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF6F8F3F-5FEB-4D1B-AF55-30D55417BBAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="3" xr2:uid="{F742BA24-48F4-444D-B408-BF74EA257E12}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="16440" activeTab="2" xr2:uid="{F742BA24-48F4-444D-B408-BF74EA257E12}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -363,13 +363,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>tsオブジェクトを変換する</t>
-    <rPh sb="9" eb="11">
-      <t>ヘンカン</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>frequencyの周期の位置を返す</t>
     <rPh sb="10" eb="12">
       <t>シュウキ</t>
@@ -1331,6 +1324,16 @@
     </rPh>
     <rPh sb="16" eb="18">
       <t>サクセイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>tsオブジェクトを要約したベクターに変換する</t>
+    <rPh sb="9" eb="11">
+      <t>ヨウヤク</t>
+    </rPh>
+    <rPh sb="18" eb="20">
+      <t>ヘンカン</t>
     </rPh>
     <phoneticPr fontId="1"/>
   </si>
@@ -1399,14 +1402,10 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office テーマ">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 テーマ">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1444,7 +1443,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1550,7 +1549,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1692,7 +1691,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1701,13 +1700,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE7181D5-8ACD-4DA3-95B3-CB4256025D66}">
   <dimension ref="A1:B20"/>
-  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="27.59765625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="48.59765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="48.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1715,7 +1714,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1723,7 +1722,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1731,7 +1730,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1739,7 +1738,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -1747,7 +1746,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -1755,7 +1754,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -1763,7 +1762,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -1771,7 +1770,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -1779,7 +1778,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -1787,7 +1786,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -1795,7 +1794,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -1803,7 +1802,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -1811,7 +1810,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>14</v>
       </c>
@@ -1819,7 +1818,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>15</v>
       </c>
@@ -1827,7 +1826,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>16</v>
       </c>
@@ -1835,7 +1834,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>17</v>
       </c>
@@ -1843,7 +1842,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>34</v>
       </c>
@@ -1851,7 +1850,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>35</v>
       </c>
@@ -1859,7 +1858,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>36</v>
       </c>
@@ -1876,302 +1875,302 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C65B167-3459-4EB0-8E33-B155F77ABBD5}">
   <dimension ref="A1:B37"/>
-  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1" t="s">
         <v>97</v>
       </c>
-      <c r="B1" t="s">
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A2" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A3" t="s">
         <v>99</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B3" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A4" t="s">
         <v>100</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B4" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A5" t="s">
         <v>101</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B5" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A6" t="s">
         <v>102</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B6" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A7" t="s">
         <v>103</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B7" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A8" t="s">
         <v>104</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B8" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A9" t="s">
+        <v>105</v>
+      </c>
+      <c r="B9" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
-        <v>105</v>
-      </c>
-      <c r="B8" t="s">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A10" t="s">
+        <v>106</v>
+      </c>
+      <c r="B10" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A9" t="s">
-        <v>106</v>
-      </c>
-      <c r="B9" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A10" t="s">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A11" t="s">
         <v>107</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B11" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A11" t="s">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A12" t="s">
         <v>108</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B12" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A13" t="s">
+        <v>109</v>
+      </c>
+      <c r="B13" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A14" t="s">
+        <v>110</v>
+      </c>
+      <c r="B14" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A12" t="s">
-        <v>109</v>
-      </c>
-      <c r="B12" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A13" t="s">
-        <v>110</v>
-      </c>
-      <c r="B13" t="s">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A15" t="s">
+        <v>111</v>
+      </c>
+      <c r="B15" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A14" t="s">
-        <v>111</v>
-      </c>
-      <c r="B14" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A15" t="s">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A16" t="s">
         <v>112</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B16" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A16" t="s">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A17" t="s">
         <v>113</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B17" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A17" t="s">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A18" t="s">
         <v>114</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B18" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A18" t="s">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A19" t="s">
         <v>115</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B19" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A19" t="s">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A20" t="s">
         <v>116</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B20" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A20" t="s">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A21" t="s">
         <v>117</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B21" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A21" t="s">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A22" t="s">
         <v>118</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B22" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A22" t="s">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A23" t="s">
+        <v>120</v>
+      </c>
+      <c r="B23" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A24" t="s">
+        <v>121</v>
+      </c>
+      <c r="B24" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A25" t="s">
+        <v>122</v>
+      </c>
+      <c r="B25" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A26" t="s">
         <v>119</v>
       </c>
-      <c r="B22" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A23" t="s">
-        <v>121</v>
-      </c>
-      <c r="B23" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A24" t="s">
-        <v>122</v>
-      </c>
-      <c r="B24" t="s">
+      <c r="B26" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A25" t="s">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A27" t="s">
         <v>123</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B27" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A28" t="s">
+        <v>124</v>
+      </c>
+      <c r="B28" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A26" t="s">
-        <v>120</v>
-      </c>
-      <c r="B26" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A27" t="s">
-        <v>124</v>
-      </c>
-      <c r="B27" t="s">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A29" t="s">
+        <v>125</v>
+      </c>
+      <c r="B29" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A30" t="s">
+        <v>126</v>
+      </c>
+      <c r="B30" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A31" t="s">
+        <v>127</v>
+      </c>
+      <c r="B31" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A28" t="s">
-        <v>125</v>
-      </c>
-      <c r="B28" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A29" t="s">
-        <v>126</v>
-      </c>
-      <c r="B29" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A30" t="s">
-        <v>127</v>
-      </c>
-      <c r="B30" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A31" t="s">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A32" t="s">
         <v>128</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B32" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A32" t="s">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A33" t="s">
         <v>129</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B33" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A34" t="s">
+        <v>130</v>
+      </c>
+      <c r="B34" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A33" t="s">
-        <v>130</v>
-      </c>
-      <c r="B33" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A34" t="s">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A35" t="s">
         <v>131</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B35" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A35" t="s">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A36" t="s">
         <v>132</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B36" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A36" t="s">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A37" t="s">
         <v>133</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B37" t="s">
         <v>168</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A37" t="s">
-        <v>134</v>
-      </c>
-      <c r="B37" t="s">
-        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -2183,13 +2182,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85ACC953-7FB5-4330-B2B4-6E3441C237F1}">
   <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="57.69921875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="57.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2197,7 +2196,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>40</v>
       </c>
@@ -2205,7 +2204,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>41</v>
       </c>
@@ -2213,7 +2212,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>42</v>
       </c>
@@ -2221,68 +2220,68 @@
         <v>53</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>43</v>
       </c>
       <c r="B5" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>44</v>
       </c>
       <c r="B6" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>45</v>
       </c>
       <c r="B7" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>46</v>
       </c>
       <c r="B8" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>47</v>
       </c>
       <c r="B9" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>48</v>
       </c>
       <c r="B10" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>49</v>
       </c>
       <c r="B11" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>50</v>
       </c>
       <c r="B12" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -2294,13 +2293,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C259549-3F86-4E62-9EDA-76EB48D3AE05}">
   <dimension ref="A1:B28"/>
-  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="22.69921875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.75" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="58" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2308,220 +2307,220 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A3" t="s">
         <v>62</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B3" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A4" t="s">
         <v>63</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B4" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A5" t="s">
         <v>64</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B5" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A6" t="s">
         <v>65</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B6" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A7" t="s">
+        <v>66</v>
+      </c>
+      <c r="B7" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A8" t="s">
+        <v>169</v>
+      </c>
+      <c r="B8" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A9" t="s">
+        <v>170</v>
+      </c>
+      <c r="B9" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A10" t="s">
+        <v>171</v>
+      </c>
+      <c r="B10" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A11" t="s">
+        <v>172</v>
+      </c>
+      <c r="B11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A12" t="s">
+        <v>173</v>
+      </c>
+      <c r="B12" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A13" t="s">
+        <v>67</v>
+      </c>
+      <c r="B13" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
-        <v>66</v>
-      </c>
-      <c r="B6" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
-        <v>67</v>
-      </c>
-      <c r="B7" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
-        <v>170</v>
-      </c>
-      <c r="B8" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A9" t="s">
-        <v>171</v>
-      </c>
-      <c r="B9" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A10" t="s">
-        <v>172</v>
-      </c>
-      <c r="B10" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A11" t="s">
-        <v>173</v>
-      </c>
-      <c r="B11" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A12" t="s">
-        <v>174</v>
-      </c>
-      <c r="B12" t="s">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A14" t="s">
+        <v>68</v>
+      </c>
+      <c r="B14" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A15" t="s">
+        <v>69</v>
+      </c>
+      <c r="B15" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A16" t="s">
+        <v>70</v>
+      </c>
+      <c r="B16" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A17" t="s">
+        <v>71</v>
+      </c>
+      <c r="B17" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A13" t="s">
-        <v>68</v>
-      </c>
-      <c r="B13" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A14" t="s">
-        <v>69</v>
-      </c>
-      <c r="B14" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A15" t="s">
-        <v>70</v>
-      </c>
-      <c r="B15" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A16" t="s">
-        <v>71</v>
-      </c>
-      <c r="B16" t="s">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A18" t="s">
+        <v>72</v>
+      </c>
+      <c r="B18" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A19" t="s">
+        <v>73</v>
+      </c>
+      <c r="B19" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A20" t="s">
+        <v>74</v>
+      </c>
+      <c r="B20" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A21" t="s">
+        <v>75</v>
+      </c>
+      <c r="B21" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A22" t="s">
+        <v>76</v>
+      </c>
+      <c r="B22" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A23" t="s">
+        <v>77</v>
+      </c>
+      <c r="B23" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A24" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A17" t="s">
-        <v>72</v>
-      </c>
-      <c r="B17" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A18" t="s">
-        <v>73</v>
-      </c>
-      <c r="B18" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A19" t="s">
-        <v>74</v>
-      </c>
-      <c r="B19" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A20" t="s">
-        <v>75</v>
-      </c>
-      <c r="B20" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A21" t="s">
-        <v>76</v>
-      </c>
-      <c r="B21" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A22" t="s">
-        <v>77</v>
-      </c>
-      <c r="B22" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A23" t="s">
+      <c r="B24" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A25" t="s">
+        <v>90</v>
+      </c>
+      <c r="B25" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A26" t="s">
         <v>78</v>
       </c>
-      <c r="B23" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A24" t="s">
-        <v>90</v>
-      </c>
-      <c r="B24" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A25" t="s">
-        <v>91</v>
-      </c>
-      <c r="B25" t="s">
+      <c r="B26" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A26" t="s">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A27" t="s">
         <v>79</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B27" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A27" t="s">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A28" t="s">
         <v>80</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B28" t="s">
         <v>95</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A28" t="s">
-        <v>81</v>
-      </c>
-      <c r="B28" t="s">
-        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>